<commit_message>
Update summarized fitur aset - KBMI 4.xlsx
</commit_message>
<xml_diff>
--- a/data/summarized fitur aset - KBMI 4.xlsx
+++ b/data/summarized fitur aset - KBMI 4.xlsx
@@ -552,10 +552,10 @@
         <v>0.01075527276849911</v>
       </c>
       <c r="M2" t="n">
-        <v>0.01657891300236998</v>
+        <v>0.6543130362564963</v>
       </c>
       <c r="N2" t="n">
-        <v>1.01602820361624</v>
+        <v>0.02574401282309871</v>
       </c>
     </row>
     <row r="3">
@@ -606,10 +606,10 @@
         <v>0.00890923687556004</v>
       </c>
       <c r="M3" t="n">
-        <v>0.02464141077589152</v>
+        <v>0.7020133223751425</v>
       </c>
       <c r="N3" t="n">
-        <v>1.062915473956672</v>
+        <v>0.03730945835216132</v>
       </c>
     </row>
     <row r="4">
@@ -660,10 +660,10 @@
         <v>0.02450315162864658</v>
       </c>
       <c r="M4" t="n">
-        <v>0.02029818009733492</v>
+        <v>0.6699885287604143</v>
       </c>
       <c r="N4" t="n">
-        <v>1.090963168889033</v>
+        <v>0.03305215825506711</v>
       </c>
     </row>
     <row r="5">
@@ -714,10 +714,10 @@
         <v>0.006957662156682413</v>
       </c>
       <c r="M5" t="n">
-        <v>0.02794918680291551</v>
+        <v>0.6400007606409356</v>
       </c>
       <c r="N5" t="n">
-        <v>1.003522863032366</v>
+        <v>0.04382439785196439</v>
       </c>
     </row>
     <row r="6">
@@ -768,10 +768,10 @@
         <v>0.00808939585906817</v>
       </c>
       <c r="M6" t="n">
-        <v>0.02719381003643478</v>
+        <v>0.5773360395628229</v>
       </c>
       <c r="N6" t="n">
-        <v>1.010969675115811</v>
+        <v>0.04761891760388536</v>
       </c>
     </row>
     <row r="7">
@@ -822,10 +822,10 @@
         <v>0.007887406245276771</v>
       </c>
       <c r="M7" t="n">
-        <v>0.04605275499795481</v>
+        <v>0.6230473013911807</v>
       </c>
       <c r="N7" t="n">
-        <v>1.031680658241608</v>
+        <v>0.07625702973761733</v>
       </c>
     </row>
     <row r="8">
@@ -876,10 +876,10 @@
         <v>0.02245901525693728</v>
       </c>
       <c r="M8" t="n">
-        <v>0.04769000277953852</v>
+        <v>0.647270856516703</v>
       </c>
       <c r="N8" t="n">
-        <v>1.037349628860651</v>
+        <v>0.07643045594536366</v>
       </c>
     </row>
     <row r="9">
@@ -930,10 +930,10 @@
         <v>0.005689154035014207</v>
       </c>
       <c r="M9" t="n">
-        <v>0.04196354137965498</v>
+        <v>0.64547614663133</v>
       </c>
       <c r="N9" t="n">
-        <v>1.058670050634366</v>
+        <v>0.06882600497175419</v>
       </c>
     </row>
     <row r="10">
@@ -984,10 +984,10 @@
         <v>0.008097578411057509</v>
       </c>
       <c r="M10" t="n">
-        <v>0.02550723165469695</v>
+        <v>0.544935047026507</v>
       </c>
       <c r="N10" t="n">
-        <v>1.023431396392182</v>
+        <v>0.04790461148151398</v>
       </c>
     </row>
     <row r="11">
@@ -1038,10 +1038,10 @@
         <v>0.008287748053300835</v>
       </c>
       <c r="M11" t="n">
-        <v>0.04837820318119871</v>
+        <v>0.6315754479570467</v>
       </c>
       <c r="N11" t="n">
-        <v>1.033625668956791</v>
+        <v>0.07917494701202332</v>
       </c>
     </row>
     <row r="12">
@@ -1092,10 +1092,10 @@
         <v>0.02651778575642104</v>
       </c>
       <c r="M12" t="n">
-        <v>0.05231951530634381</v>
+        <v>0.674368266412619</v>
       </c>
       <c r="N12" t="n">
-        <v>1.036881400117148</v>
+        <v>0.08044437288379079</v>
       </c>
     </row>
     <row r="13">
@@ -1146,10 +1146,10 @@
         <v>0.004764252658911321</v>
       </c>
       <c r="M13" t="n">
-        <v>0.04510475612294877</v>
+        <v>0.6194223167806974</v>
       </c>
       <c r="N13" t="n">
-        <v>1.036091072678112</v>
+        <v>0.07544551413192954</v>
       </c>
     </row>
     <row r="14">
@@ -1200,10 +1200,10 @@
         <v>0.009826595588117137</v>
       </c>
       <c r="M14" t="n">
-        <v>0.02754209810427008</v>
+        <v>0.5357667436378493</v>
       </c>
       <c r="N14" t="n">
-        <v>1.035906784083837</v>
+        <v>0.05325273845926031</v>
       </c>
     </row>
     <row r="15">
@@ -1254,10 +1254,10 @@
         <v>0.007995493336151174</v>
       </c>
       <c r="M15" t="n">
-        <v>0.04788172130255296</v>
+        <v>0.6214711828178504</v>
       </c>
       <c r="N15" t="n">
-        <v>1.026814076317421</v>
+        <v>0.07911167370439323</v>
       </c>
     </row>
     <row r="16">
@@ -1308,10 +1308,10 @@
         <v>0.02484901372153656</v>
       </c>
       <c r="M16" t="n">
-        <v>0.05488417536485788</v>
+        <v>0.6641789343593151</v>
       </c>
       <c r="N16" t="n">
-        <v>1.027789865675865</v>
+        <v>0.08493102732984435</v>
       </c>
     </row>
     <row r="17">
@@ -1362,10 +1362,10 @@
         <v>0.003918431706350286</v>
       </c>
       <c r="M17" t="n">
-        <v>0.05188224801669713</v>
+        <v>0.6523125705398802</v>
       </c>
       <c r="N17" t="n">
-        <v>1.027678657225814</v>
+        <v>0.08173731640880014</v>
       </c>
     </row>
     <row r="18">
@@ -1416,10 +1416,10 @@
         <v>0.009995710124041378</v>
       </c>
       <c r="M18" t="n">
-        <v>0.02877990352133709</v>
+        <v>0.5226731350776493</v>
       </c>
       <c r="N18" t="n">
-        <v>1.022842504629262</v>
+        <v>0.05632068423868711</v>
       </c>
     </row>
     <row r="19">
@@ -1470,10 +1470,10 @@
         <v>0.006792190309852888</v>
       </c>
       <c r="M19" t="n">
-        <v>0.04868571576224905</v>
+        <v>0.6509184930744206</v>
       </c>
       <c r="N19" t="n">
-        <v>1.026380902133355</v>
+        <v>0.07676858070055186</v>
       </c>
     </row>
     <row r="20">
@@ -1524,10 +1524,10 @@
         <v>0.02424449042911652</v>
       </c>
       <c r="M20" t="n">
-        <v>0.05661926532116838</v>
+        <v>0.666907467483271</v>
       </c>
       <c r="N20" t="n">
-        <v>1.029778324082162</v>
+        <v>0.0874263597215735</v>
       </c>
     </row>
     <row r="21">
@@ -1578,10 +1578,10 @@
         <v>0.004013426982055066</v>
       </c>
       <c r="M21" t="n">
-        <v>0.05458174171201331</v>
+        <v>0.6461226034051759</v>
       </c>
       <c r="N21" t="n">
-        <v>1.031571564638912</v>
+        <v>0.08714286174456946</v>
       </c>
     </row>
     <row r="22">
@@ -1632,10 +1632,10 @@
         <v>0.01092964117340185</v>
       </c>
       <c r="M22" t="n">
-        <v>0.0279850854585897</v>
+        <v>0.5147438455478128</v>
       </c>
       <c r="N22" t="n">
-        <v>1.02066364081003</v>
+        <v>0.05549043365860082</v>
       </c>
     </row>
     <row r="23">
@@ -1686,10 +1686,10 @@
         <v>0.006378200131800918</v>
       </c>
       <c r="M23" t="n">
-        <v>0.04740124255771754</v>
+        <v>0.6302898941181441</v>
       </c>
       <c r="N23" t="n">
-        <v>1.025242039915222</v>
+        <v>0.07710380107297292</v>
       </c>
     </row>
     <row r="24">
@@ -1740,10 +1740,10 @@
         <v>0.02397144620800645</v>
       </c>
       <c r="M24" t="n">
-        <v>0.05503027287942899</v>
+        <v>0.6364648560376018</v>
       </c>
       <c r="N24" t="n">
-        <v>1.040442772591639</v>
+        <v>0.08995916922672152</v>
       </c>
     </row>
     <row r="25">
@@ -1794,10 +1794,10 @@
         <v>0.003770883875911295</v>
       </c>
       <c r="M25" t="n">
-        <v>0.05171079951746201</v>
+        <v>0.6051617678611098</v>
       </c>
       <c r="N25" t="n">
-        <v>1.023041561308376</v>
+        <v>0.08741843897678331</v>
       </c>
     </row>
     <row r="26">
@@ -1848,10 +1848,10 @@
         <v>0.009506754014840047</v>
       </c>
       <c r="M26" t="n">
-        <v>0.0267024554017725</v>
+        <v>0.5148439288552971</v>
       </c>
       <c r="N26" t="n">
-        <v>1.025678642515216</v>
+        <v>0.05319697227314662</v>
       </c>
     </row>
     <row r="27">
@@ -1902,10 +1902,10 @@
         <v>0.007548074914001441</v>
       </c>
       <c r="M27" t="n">
-        <v>0.04462248711454708</v>
+        <v>0.6109036624659336</v>
       </c>
       <c r="N27" t="n">
-        <v>1.028851647760216</v>
+        <v>0.07515083345489169</v>
       </c>
     </row>
     <row r="28">
@@ -1956,10 +1956,10 @@
         <v>0.02290393659689072</v>
       </c>
       <c r="M28" t="n">
-        <v>0.05334943511207615</v>
+        <v>0.6178181193369826</v>
       </c>
       <c r="N28" t="n">
-        <v>1.033240421291009</v>
+        <v>0.08922171604483611</v>
       </c>
     </row>
     <row r="29">
@@ -2010,10 +2010,10 @@
         <v>0.006015966055517137</v>
       </c>
       <c r="M29" t="n">
-        <v>0.05144533161708193</v>
+        <v>0.6000292937064021</v>
       </c>
       <c r="N29" t="n">
-        <v>1.024187315051129</v>
+        <v>0.08781180621257377</v>
       </c>
     </row>
     <row r="30">
@@ -2064,10 +2064,10 @@
         <v>0.01119446144101002</v>
       </c>
       <c r="M30" t="n">
-        <v>0.02830527814822404</v>
+        <v>0.5022021513820725</v>
       </c>
       <c r="N30" t="n">
-        <v>1.01499278114327</v>
+        <v>0.05720734749868165</v>
       </c>
     </row>
     <row r="31">
@@ -2118,10 +2118,10 @@
         <v>0.007940750188881679</v>
       </c>
       <c r="M31" t="n">
-        <v>0.04513223240318735</v>
+        <v>0.6226510431513592</v>
       </c>
       <c r="N31" t="n">
-        <v>1.027406047455745</v>
+        <v>0.07447049035930227</v>
       </c>
     </row>
     <row r="32">
@@ -2172,10 +2172,10 @@
         <v>0.02391611789032971</v>
       </c>
       <c r="M32" t="n">
-        <v>0.05632285933962994</v>
+        <v>0.6503826320204547</v>
       </c>
       <c r="N32" t="n">
-        <v>1.038904108989339</v>
+        <v>0.08996865401554859</v>
       </c>
     </row>
     <row r="33">
@@ -2226,10 +2226,10 @@
         <v>0.005552587155284447</v>
       </c>
       <c r="M33" t="n">
-        <v>0.05498882336282065</v>
+        <v>0.6326363863308309</v>
       </c>
       <c r="N33" t="n">
-        <v>1.024873201144919</v>
+        <v>0.08908208987773174</v>
       </c>
     </row>
     <row r="34">
@@ -2280,10 +2280,10 @@
         <v>0.01179289987700865</v>
       </c>
       <c r="M34" t="n">
-        <v>0.02886096791604882</v>
+        <v>0.5307188364495358</v>
       </c>
       <c r="N34" t="n">
-        <v>1.016772674802146</v>
+        <v>0.0552930130418881</v>
       </c>
     </row>
     <row r="35">
@@ -2334,10 +2334,10 @@
         <v>0.009183777834109997</v>
       </c>
       <c r="M35" t="n">
-        <v>0.04291998663929377</v>
+        <v>0.6395328479974554</v>
       </c>
       <c r="N35" t="n">
-        <v>1.02901514775923</v>
+        <v>0.06905871454726716</v>
       </c>
     </row>
     <row r="36">
@@ -2388,10 +2388,10 @@
         <v>0.02516709661982215</v>
       </c>
       <c r="M36" t="n">
-        <v>0.05614837741546663</v>
+        <v>0.6755343506418707</v>
       </c>
       <c r="N36" t="n">
-        <v>1.037791236013939</v>
+        <v>0.08625807694724584</v>
       </c>
     </row>
     <row r="37">
@@ -2442,10 +2442,10 @@
         <v>0.005218418746152272</v>
       </c>
       <c r="M37" t="n">
-        <v>0.05731101131233773</v>
+        <v>0.6505184530864599</v>
       </c>
       <c r="N37" t="n">
-        <v>1.021444066634962</v>
+        <v>0.08998974922246523</v>
       </c>
     </row>
     <row r="38">
@@ -2496,10 +2496,10 @@
         <v>0.01217253025992921</v>
       </c>
       <c r="M38" t="n">
-        <v>0.02819437348695034</v>
+        <v>0.5261440302474134</v>
       </c>
       <c r="N38" t="n">
-        <v>1.016808194376687</v>
+        <v>0.05448749458084125</v>
       </c>
     </row>
     <row r="39">
@@ -2550,10 +2550,10 @@
         <v>0.005991101878336911</v>
       </c>
       <c r="M39" t="n">
-        <v>0.04125296286539953</v>
+        <v>0.6290993015103593</v>
       </c>
       <c r="N39" t="n">
-        <v>1.029701327673346</v>
+        <v>0.06752229819835787</v>
       </c>
     </row>
     <row r="40">
@@ -2604,10 +2604,10 @@
         <v>0.02311670420668254</v>
       </c>
       <c r="M40" t="n">
-        <v>0.05607961913958524</v>
+        <v>0.6805225035579979</v>
       </c>
       <c r="N40" t="n">
-        <v>1.044107614278077</v>
+        <v>0.0860414711391911</v>
       </c>
     </row>
     <row r="41">
@@ -2658,10 +2658,10 @@
         <v>0.00539015919188091</v>
       </c>
       <c r="M41" t="n">
-        <v>0.05532606299121029</v>
+        <v>0.6391316572842384</v>
       </c>
       <c r="N41" t="n">
-        <v>1.02532580207194</v>
+        <v>0.08875673621455007</v>
       </c>
     </row>
     <row r="42">
@@ -2712,10 +2712,10 @@
         <v>0.01208937567948008</v>
       </c>
       <c r="M42" t="n">
-        <v>0.02640916591583858</v>
+        <v>0.5385378362985057</v>
       </c>
       <c r="N42" t="n">
-        <v>1.017351350817073</v>
+        <v>0.0498895320022385</v>
       </c>
     </row>
     <row r="43">
@@ -2766,10 +2766,10 @@
         <v>0.007232788062864638</v>
       </c>
       <c r="M43" t="n">
-        <v>0.0345579245808216</v>
+        <v>0.5939119966883081</v>
       </c>
       <c r="N43" t="n">
-        <v>1.031926229324679</v>
+        <v>0.06004463456677625</v>
       </c>
     </row>
     <row r="44">
@@ -2820,10 +2820,10 @@
         <v>0.02001939544604218</v>
       </c>
       <c r="M44" t="n">
-        <v>0.0503031342533605</v>
+        <v>0.6442035187594678</v>
       </c>
       <c r="N44" t="n">
-        <v>1.030352826559046</v>
+        <v>0.08045590415671325</v>
       </c>
     </row>
     <row r="45">
@@ -2874,10 +2874,10 @@
         <v>0.004052964357590595</v>
       </c>
       <c r="M45" t="n">
-        <v>0.04830329886446205</v>
+        <v>0.5881243186397747</v>
       </c>
       <c r="N45" t="n">
-        <v>1.022082869234672</v>
+        <v>0.08394479318772788</v>
       </c>
     </row>
     <row r="46">
@@ -2928,10 +2928,10 @@
         <v>0.01006533674794197</v>
       </c>
       <c r="M46" t="n">
-        <v>0.02699293560057618</v>
+        <v>0.5382738075577017</v>
       </c>
       <c r="N46" t="n">
-        <v>1.01487772998211</v>
+        <v>0.05089329784067081</v>
       </c>
     </row>
     <row r="47">
@@ -2982,10 +2982,10 @@
         <v>0.00795295246756814</v>
       </c>
       <c r="M47" t="n">
-        <v>0.03574869180797206</v>
+        <v>0.629111779390783</v>
       </c>
       <c r="N47" t="n">
-        <v>1.034494574704442</v>
+        <v>0.05878419215729921</v>
       </c>
     </row>
     <row r="48">
@@ -3036,10 +3036,10 @@
         <v>0.01768928650069429</v>
       </c>
       <c r="M48" t="n">
-        <v>0.05111630492553221</v>
+        <v>0.6432080485751298</v>
       </c>
       <c r="N48" t="n">
-        <v>1.022908704464536</v>
+        <v>0.08129144740060401</v>
       </c>
     </row>
     <row r="49">
@@ -3090,10 +3090,10 @@
         <v>0.004754168156210271</v>
       </c>
       <c r="M49" t="n">
-        <v>0.05083306336915244</v>
+        <v>0.6267809953593146</v>
       </c>
       <c r="N49" t="n">
-        <v>1.023327534666394</v>
+        <v>0.08299369923823946</v>
       </c>
     </row>
     <row r="50">
@@ -3144,10 +3144,10 @@
         <v>0.0100136610160599</v>
       </c>
       <c r="M50" t="n">
-        <v>0.02619691316701024</v>
+        <v>0.5405245177302375</v>
       </c>
       <c r="N50" t="n">
-        <v>1.015644640848093</v>
+        <v>0.04922395486621679</v>
       </c>
     </row>
     <row r="51">
@@ -3198,10 +3198,10 @@
         <v>0.006195471490433611</v>
       </c>
       <c r="M51" t="n">
-        <v>0.03348213887675885</v>
+        <v>0.6443648955627385</v>
       </c>
       <c r="N51" t="n">
-        <v>1.049006243276712</v>
+        <v>0.05450789290640089</v>
       </c>
     </row>
     <row r="52">
@@ -3252,10 +3252,10 @@
         <v>0.01797350990008636</v>
       </c>
       <c r="M52" t="n">
-        <v>0.0493515816878574</v>
+        <v>0.6520427595006858</v>
       </c>
       <c r="N52" t="n">
-        <v>1.020771413079048</v>
+        <v>0.07725978556341484</v>
       </c>
     </row>
     <row r="53">
@@ -3306,10 +3306,10 @@
         <v>0.004521622380496413</v>
       </c>
       <c r="M53" t="n">
-        <v>0.0474485143699144</v>
+        <v>0.646602237457938</v>
       </c>
       <c r="N53" t="n">
-        <v>1.032827671412701</v>
+        <v>0.07579023976368264</v>
       </c>
     </row>
     <row r="54">
@@ -3360,10 +3360,10 @@
         <v>0.009801839037172848</v>
       </c>
       <c r="M54" t="n">
-        <v>0.02557367741508091</v>
+        <v>0.5526281768569941</v>
       </c>
       <c r="N54" t="n">
-        <v>1.014443035613116</v>
+        <v>0.0469448356692436</v>
       </c>
     </row>
     <row r="55">
@@ -3414,10 +3414,10 @@
         <v>0.008166697929512988</v>
       </c>
       <c r="M55" t="n">
-        <v>0.02994685996667913</v>
+        <v>0.6515018816757246</v>
       </c>
       <c r="N55" t="n">
-        <v>1.053583006591842</v>
+        <v>0.04842887434265763</v>
       </c>
     </row>
     <row r="56">
@@ -3468,10 +3468,10 @@
         <v>0.02101080373134009</v>
       </c>
       <c r="M56" t="n">
-        <v>0.05039723977149593</v>
+        <v>0.6845072682917085</v>
       </c>
       <c r="N56" t="n">
-        <v>1.021087512869041</v>
+        <v>0.07517815310006526</v>
       </c>
     </row>
     <row r="57">
@@ -3522,10 +3522,10 @@
         <v>0.005246835801358314</v>
       </c>
       <c r="M57" t="n">
-        <v>0.04623179573185095</v>
+        <v>0.6581686870837286</v>
       </c>
       <c r="N57" t="n">
-        <v>1.041345740871147</v>
+        <v>0.07314733217027589</v>
       </c>
     </row>
     <row r="58">
@@ -3576,10 +3576,10 @@
         <v>0.01090017927646798</v>
       </c>
       <c r="M58" t="n">
-        <v>0.0241951959563715</v>
+        <v>0.5744518806230234</v>
       </c>
       <c r="N58" t="n">
-        <v>1.022453357917308</v>
+        <v>0.04306445880937693</v>
       </c>
     </row>
     <row r="59">
@@ -3630,10 +3630,10 @@
         <v>0.008563778726911917</v>
       </c>
       <c r="M59" t="n">
-        <v>0.02506055147093447</v>
+        <v>0.6429151076043956</v>
       </c>
       <c r="N59" t="n">
-        <v>1.038630693352978</v>
+        <v>0.04048537301767816</v>
       </c>
     </row>
     <row r="60">
@@ -3684,10 +3684,10 @@
         <v>0.01672962581950657</v>
       </c>
       <c r="M60" t="n">
-        <v>0.04474508614777217</v>
+        <v>0.6559508518665338</v>
       </c>
       <c r="N60" t="n">
-        <v>1.035307418129013</v>
+        <v>0.07062254661578822</v>
       </c>
     </row>
     <row r="61">
@@ -3738,10 +3738,10 @@
         <v>0.005567315115064913</v>
       </c>
       <c r="M61" t="n">
-        <v>0.04196155469239227</v>
+        <v>0.624483475531688</v>
       </c>
       <c r="N61" t="n">
-        <v>1.034409606350561</v>
+        <v>0.06950613902835369</v>
       </c>
     </row>
     <row r="62">
@@ -3792,10 +3792,10 @@
         <v>0.0107056836999868</v>
       </c>
       <c r="M62" t="n">
-        <v>0.02395656693500777</v>
+        <v>0.577684291467868</v>
       </c>
       <c r="N62" t="n">
-        <v>1.021684864534631</v>
+        <v>0.04236927021421293</v>
       </c>
     </row>
     <row r="63">
@@ -3846,10 +3846,10 @@
         <v>0.007966651671683329</v>
       </c>
       <c r="M63" t="n">
-        <v>0.0248565479887341</v>
+        <v>0.6684184821005454</v>
       </c>
       <c r="N63" t="n">
-        <v>1.038129326317226</v>
+        <v>0.03860502381236487</v>
       </c>
     </row>
     <row r="64">
@@ -3900,10 +3900,10 @@
         <v>0.01834081208076097</v>
       </c>
       <c r="M64" t="n">
-        <v>0.0449213399114869</v>
+        <v>0.6684746760007089</v>
       </c>
       <c r="N64" t="n">
-        <v>1.033006752651791</v>
+        <v>0.06941780912981535</v>
       </c>
     </row>
     <row r="65">
@@ -3954,10 +3954,10 @@
         <v>0.00576964869262816</v>
       </c>
       <c r="M65" t="n">
-        <v>0.04229137955445521</v>
+        <v>0.6385413852111044</v>
       </c>
       <c r="N65" t="n">
-        <v>1.029607306005856</v>
+        <v>0.06819215540107572</v>
       </c>
     </row>
     <row r="66">
@@ -4008,10 +4008,10 @@
         <v>0.008665843262894261</v>
       </c>
       <c r="M66" t="n">
-        <v>0.02423318318175136</v>
+        <v>0.5953839958631545</v>
       </c>
       <c r="N66" t="n">
-        <v>1.027204077433941</v>
+        <v>0.04180902534575347</v>
       </c>
     </row>
     <row r="67">
@@ -4062,10 +4062,10 @@
         <v>0.008642455342039206</v>
       </c>
       <c r="M67" t="n">
-        <v>0.0227176804227838</v>
+        <v>0.6805589086326084</v>
       </c>
       <c r="N67" t="n">
-        <v>1.04135334400671</v>
+        <v>0.03476132951352298</v>
       </c>
     </row>
     <row r="68">
@@ -4116,10 +4116,10 @@
         <v>0.01882272518071008</v>
       </c>
       <c r="M68" t="n">
-        <v>0.04100718952865304</v>
+        <v>0.6947127364122128</v>
       </c>
       <c r="N68" t="n">
-        <v>1.028838851958299</v>
+        <v>0.06072983491648868</v>
       </c>
     </row>
     <row r="69">
@@ -4170,10 +4170,10 @@
         <v>0.005622437317282039</v>
       </c>
       <c r="M69" t="n">
-        <v>0.04238300177405969</v>
+        <v>0.658595497597406</v>
       </c>
       <c r="N69" t="n">
-        <v>1.017048236066221</v>
+        <v>0.06545073167179316</v>
       </c>
     </row>
     <row r="70">
@@ -4224,10 +4224,10 @@
         <v>0.007313845262303325</v>
       </c>
       <c r="M70" t="n">
-        <v>0.02438689336590067</v>
+        <v>0.6111582780281156</v>
       </c>
       <c r="N70" t="n">
-        <v>1.02515329214211</v>
+        <v>0.04090643114551996</v>
       </c>
     </row>
     <row r="71">
@@ -4278,10 +4278,10 @@
         <v>0.005962867759101964</v>
       </c>
       <c r="M71" t="n">
-        <v>0.02111454242546383</v>
+        <v>0.686145116928202</v>
       </c>
       <c r="N71" t="n">
-        <v>1.04054332577815</v>
+        <v>0.03202033455551791</v>
       </c>
     </row>
     <row r="72">
@@ -4332,10 +4332,10 @@
         <v>0.0147517042506812</v>
       </c>
       <c r="M72" t="n">
-        <v>0.03960597768448311</v>
+        <v>0.7060645338951592</v>
       </c>
       <c r="N72" t="n">
-        <v>1.025564474970187</v>
+        <v>0.0575280045374707</v>
       </c>
     </row>
     <row r="73">
@@ -4386,10 +4386,10 @@
         <v>0.005701168764623488</v>
       </c>
       <c r="M73" t="n">
-        <v>0.04152698077250187</v>
+        <v>0.6724674463159386</v>
       </c>
       <c r="N73" t="n">
-        <v>1.021086692399422</v>
+        <v>0.06305531617125558</v>
       </c>
     </row>
     <row r="74">
@@ -4440,10 +4440,10 @@
         <v>0.007154610075165223</v>
       </c>
       <c r="M74" t="n">
-        <v>0.02302589615015578</v>
+        <v>0.6363457737501406</v>
       </c>
       <c r="N74" t="n">
-        <v>1.028619104078975</v>
+        <v>0.03722013667036401</v>
       </c>
     </row>
     <row r="75">
@@ -4494,10 +4494,10 @@
         <v>0.004880208795921642</v>
       </c>
       <c r="M75" t="n">
-        <v>0.02037882504109474</v>
+        <v>0.698217776871347</v>
       </c>
       <c r="N75" t="n">
-        <v>1.037792427760322</v>
+        <v>0.03028996255160867</v>
       </c>
     </row>
     <row r="76">
@@ -4548,10 +4548,10 @@
         <v>0.01475696250557815</v>
       </c>
       <c r="M76" t="n">
-        <v>0.03534464027170819</v>
+        <v>0.7022621127599681</v>
       </c>
       <c r="N76" t="n">
-        <v>1.030815764010355</v>
+        <v>0.05188064641870414</v>
       </c>
     </row>
     <row r="77">
@@ -4602,10 +4602,10 @@
         <v>0.005490871614548416</v>
       </c>
       <c r="M77" t="n">
-        <v>0.03866660724536687</v>
+        <v>0.6606446945903861</v>
       </c>
       <c r="N77" t="n">
-        <v>1.020392855816404</v>
+        <v>0.05972216247993057</v>
       </c>
     </row>
   </sheetData>

</xml_diff>